<commit_message>
Calibration corrections; BHRaSYC temp fix
</commit_message>
<xml_diff>
--- a/InputData/fuels/FSPbPPT/Fuel Surcharge Perc by Power Plant Type.xlsx
+++ b/InputData/fuels/FSPbPPT/Fuel Surcharge Perc by Power Plant Type.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmahajan\Documents\eps-us\InputData\fuels\FSPbPPT\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mary Francis Swint\Vensim\eps-indonesia\InputData\fuels\FSPbPPT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65263F8A-FDBA-4D8E-81F2-4CDEE15290AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E05F9FF-0352-4D90-A1D4-F533AB0E992C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" tabRatio="730" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-5880" windowWidth="38640" windowHeight="21120" tabRatio="730" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -541,69 +541,69 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="107" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B3" s="4"/>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B5" s="2"/>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B7" s="3"/>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>28</v>
       </c>
@@ -620,13 +620,13 @@
     <tabColor theme="8" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:B25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="36.28515625" customWidth="1"/>
-    <col min="2" max="2" width="29.140625" customWidth="1"/>
+    <col min="1" max="1" width="36.26953125" customWidth="1"/>
+    <col min="2" max="2" width="29.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>19</v>
       </c>
@@ -634,7 +634,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -642,7 +642,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -650,7 +650,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -658,7 +658,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -666,7 +666,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -674,7 +674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -682,7 +682,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -690,7 +690,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -698,7 +698,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>5</v>
       </c>
@@ -706,7 +706,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>6</v>
       </c>
@@ -714,7 +714,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>7</v>
       </c>
@@ -722,15 +722,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>8</v>
       </c>
       <c r="B13">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>10</v>
       </c>
@@ -738,7 +738,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>11</v>
       </c>
@@ -746,7 +746,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -754,7 +754,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -762,7 +762,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -770,7 +770,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>30</v>
       </c>
@@ -778,7 +778,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>31</v>
       </c>
@@ -786,7 +786,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>32</v>
       </c>
@@ -794,7 +794,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>33</v>
       </c>
@@ -802,7 +802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>34</v>
       </c>
@@ -810,7 +810,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" s="8" t="s">
         <v>35</v>
       </c>
@@ -818,7 +818,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" s="8" t="s">
         <v>36</v>
       </c>
@@ -977,6 +977,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -985,20 +991,37 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC1D71BC-5147-4793-AF84-07D3CFED082B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="1659011e-6b88-4225-9a61-aaf33aaf19e8"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC1D71BC-5147-4793-AF84-07D3CFED082B}"/>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CE4AAF61-7CFA-46B8-BB2B-7108BC9B9B64}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{568DE7F3-FEB2-4BF6-A999-67F40BACA2C2}"/>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CE4AAF61-7CFA-46B8-BB2B-7108BC9B9B64}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{568DE7F3-FEB2-4BF6-A999-67F40BACA2C2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>